<commit_message>
data cleaning and made two graphs
</commit_message>
<xml_diff>
--- a/data/raw/home_affairs_italians.xlsx
+++ b/data/raw/home_affairs_italians.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chloe\Downloads\S2 2026\FIT3179\coffee-visualisation\coffee-visualisation\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chloe\Downloads\S2 2026\FIT3179\coffee-visualisation\coffee-visualisation\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1440CB4A-17AA-4091-AC1A-03985396793D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1748B22-AB0E-4967-B080-EA29AE637B87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11190" yWindow="0" windowWidth="11460" windowHeight="14410" xr2:uid="{6BC50AFD-A1DA-4A83-994E-4CED1A59DD18}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6BC50AFD-A1DA-4A83-994E-4CED1A59DD18}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="8">
   <si>
     <t>Rank</t>
   </si>
@@ -59,19 +59,10 @@
     <t>Total overseas born</t>
   </si>
   <si>
-    <t>Total population (a)</t>
-  </si>
-  <si>
     <t>Census Year</t>
   </si>
   <si>
     <t>Total population</t>
-  </si>
-  <si>
-    <t>Total population (b) (c)</t>
-  </si>
-  <si>
-    <t>Total population (c) (d)</t>
   </si>
 </sst>
 </file>
@@ -444,11 +435,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40464B88-09BD-4E3F-9205-001A2063C2F1}">
   <dimension ref="A1:E34"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -460,12 +451,12 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>10</v>
+        <v>1901</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
@@ -477,37 +468,34 @@
         <v>0.7</v>
       </c>
       <c r="E2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
         <v>1901</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>5</v>
       </c>
       <c r="C3">
         <v>857576</v>
       </c>
-      <c r="D3">
-        <v>100</v>
-      </c>
-      <c r="E3">
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
         <v>1901</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C4">
         <v>3788123</v>
       </c>
-      <c r="E4">
-        <v>1901</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>6</v>
+        <v>1911</v>
       </c>
       <c r="B5" t="s">
         <v>4</v>
@@ -519,37 +507,34 @@
         <v>0.9</v>
       </c>
       <c r="E5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
         <v>1911</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>5</v>
       </c>
       <c r="C6">
         <v>756865</v>
       </c>
-      <c r="D6">
-        <v>100</v>
-      </c>
-      <c r="E6">
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7">
         <v>1911</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C7">
         <v>4455005</v>
       </c>
-      <c r="E7">
-        <v>1911</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>6</v>
+        <v>1921</v>
       </c>
       <c r="B8" t="s">
         <v>4</v>
@@ -561,37 +546,34 @@
         <v>1</v>
       </c>
       <c r="E8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9">
         <v>1921</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>5</v>
       </c>
       <c r="C9">
         <v>839579</v>
       </c>
-      <c r="D9">
-        <v>100</v>
-      </c>
-      <c r="E9">
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10">
         <v>1921</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C10">
         <v>5455136</v>
       </c>
-      <c r="E10">
-        <v>1921</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>4</v>
+        <v>1933</v>
       </c>
       <c r="B11" t="s">
         <v>4</v>
@@ -603,37 +585,34 @@
         <v>3</v>
       </c>
       <c r="E11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12">
         <v>1933</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>5</v>
       </c>
       <c r="C12">
         <v>903273</v>
       </c>
-      <c r="D12">
-        <v>100</v>
-      </c>
-      <c r="E12">
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13">
         <v>1933</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C13">
         <v>6629836</v>
       </c>
-      <c r="E13">
-        <v>1933</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>4</v>
+        <v>1947</v>
       </c>
       <c r="B14" t="s">
         <v>4</v>
@@ -645,37 +624,34 @@
         <v>4.5</v>
       </c>
       <c r="E14">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15">
         <v>1947</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>5</v>
       </c>
       <c r="C15">
         <v>744187</v>
       </c>
-      <c r="D15">
-        <v>100</v>
-      </c>
-      <c r="E15">
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16">
         <v>1947</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C16">
         <v>7579358</v>
       </c>
-      <c r="E16">
-        <v>1947</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>2</v>
+        <v>1954</v>
       </c>
       <c r="B17" t="s">
         <v>4</v>
@@ -687,37 +663,34 @@
         <v>9.3000000000000007</v>
       </c>
       <c r="E17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18">
         <v>1954</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
         <v>5</v>
       </c>
       <c r="C18">
         <v>1286466</v>
       </c>
-      <c r="D18">
-        <v>100</v>
-      </c>
-      <c r="E18">
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19">
         <v>1954</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B19" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C19">
         <v>8986530</v>
       </c>
-      <c r="E19">
-        <v>1954</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>2</v>
+        <v>1961</v>
       </c>
       <c r="B20" t="s">
         <v>4</v>
@@ -729,37 +702,34 @@
         <v>12.8</v>
       </c>
       <c r="E20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21">
         <v>1961</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B21" t="s">
         <v>5</v>
       </c>
       <c r="C21">
         <v>1778780</v>
       </c>
-      <c r="D21">
-        <v>100</v>
-      </c>
-      <c r="E21">
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22">
         <v>1961</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B22" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C22">
         <v>10508186</v>
       </c>
-      <c r="E22">
-        <v>1961</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23">
-        <v>2</v>
+        <v>1971</v>
       </c>
       <c r="B23" t="s">
         <v>4</v>
@@ -771,37 +741,34 @@
         <v>11.2</v>
       </c>
       <c r="E23">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24">
         <v>1971</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B24" t="s">
         <v>5</v>
       </c>
       <c r="C24">
         <v>2579318</v>
       </c>
-      <c r="D24">
-        <v>100</v>
-      </c>
-      <c r="E24">
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25">
         <v>1971</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B25" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C25">
         <v>12755638</v>
       </c>
-      <c r="E25">
-        <v>1971</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>2</v>
+        <v>1981</v>
       </c>
       <c r="B26" t="s">
         <v>4</v>
@@ -813,37 +780,34 @@
         <v>9.3000000000000007</v>
       </c>
       <c r="E26">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27">
         <v>1981</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>5</v>
       </c>
       <c r="C27">
         <v>2973834</v>
       </c>
-      <c r="D27">
-        <v>100</v>
-      </c>
-      <c r="E27">
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28">
         <v>1981</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B28" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C28">
         <v>17752824</v>
       </c>
-      <c r="E28">
-        <v>1981</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29">
-        <v>3</v>
+        <v>1991</v>
       </c>
       <c r="B29" t="s">
         <v>4</v>
@@ -855,37 +819,34 @@
         <v>6.9</v>
       </c>
       <c r="E29">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30">
         <v>1991</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B30" t="s">
         <v>5</v>
       </c>
       <c r="C30">
         <v>3689128</v>
       </c>
-      <c r="D30">
-        <v>100</v>
-      </c>
-      <c r="E30">
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31">
         <v>1991</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B31" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C31">
         <v>16770635</v>
       </c>
-      <c r="E31">
-        <v>1991</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32">
-        <v>3</v>
+        <v>2001</v>
       </c>
       <c r="B32" t="s">
         <v>4</v>
@@ -897,32 +858,29 @@
         <v>5.3</v>
       </c>
       <c r="E32">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33">
         <v>2001</v>
       </c>
-    </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B33" t="s">
         <v>5</v>
       </c>
       <c r="C33">
         <v>4105468</v>
       </c>
-      <c r="D33">
-        <v>100</v>
-      </c>
-      <c r="E33">
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34">
         <v>2001</v>
       </c>
-    </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B34" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C34">
         <v>18769249</v>
-      </c>
-      <c r="E34">
-        <v>2001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>